<commit_message>
changed PB with latch version , added lates CM5 image file
</commit_message>
<xml_diff>
--- a/Hardware/Manufacturing Files/BOM/Network Analyzer.xlsx
+++ b/Hardware/Manufacturing Files/BOM/Network Analyzer.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="28800" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="Network Analyzer" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="137">
   <si>
     <t>Item</t>
   </si>
@@ -206,7 +206,10 @@
     <t>PB400OAQR1BLK:SW_PB400OAQR1BLK</t>
   </si>
   <si>
-    <t>PUSHBUTTON, 3A, 30VDC DPST, Off-(On), Through Hole, Right Angle</t>
+    <t>PB400EEQR1BLK</t>
+  </si>
+  <si>
+    <t>Pushbutton Switch DPST Standard Through Hole, Right Angle</t>
   </si>
   <si>
     <t>R1,R2</t>
@@ -608,18 +611,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -961,7 +958,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -985,16 +982,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1003,85 +1000,85 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1104,7 +1101,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2012,10 +2009,10 @@
         <v>58</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H16" s="2"/>
     </row>
@@ -2024,16 +2021,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C17" s="4">
         <v>2</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -2044,16 +2041,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="C18" s="4">
-        <v>1</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>62</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -2064,20 +2061,20 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C19" s="4">
         <v>1</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H19" s="2"/>
     </row>
@@ -2086,20 +2083,20 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C20" s="4">
         <v>2</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H20" s="2"/>
     </row>
@@ -2108,20 +2105,20 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C21" s="4">
         <v>1</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H21" s="2"/>
     </row>
@@ -2130,7 +2127,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C22" s="4">
         <v>1</v>
@@ -2139,11 +2136,11 @@
         <v>100</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H22" s="2"/>
     </row>
@@ -2152,7 +2149,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C23" s="4">
         <v>2</v>
@@ -2161,11 +2158,11 @@
         <v>10</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -2174,20 +2171,20 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C24" s="4">
         <v>2</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H24" s="2"/>
     </row>
@@ -2196,20 +2193,20 @@
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C25" s="4">
         <v>1</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H25" s="2"/>
     </row>
@@ -2218,7 +2215,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C26" s="4">
         <v>1</v>
@@ -2227,13 +2224,13 @@
         <v>1040310811</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F26" s="4">
         <v>1040310811</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H26" s="2"/>
     </row>
@@ -2242,22 +2239,22 @@
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C27" s="4">
         <v>1</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E27" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F27" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="F27" s="4" t="s">
-        <v>82</v>
-      </c>
       <c r="G27" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H27" s="2"/>
     </row>
@@ -2266,22 +2263,22 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C28" s="4">
         <v>1</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H28" s="2"/>
     </row>
@@ -2290,19 +2287,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C29" s="4">
         <v>2</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="2"/>
@@ -2312,22 +2309,22 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C30" s="4">
         <v>1</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H30" s="2"/>
     </row>
@@ -2336,22 +2333,22 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C31" s="4">
         <v>1</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E31" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>100</v>
-      </c>
       <c r="G31" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H31" s="2"/>
     </row>
@@ -2360,22 +2357,22 @@
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C32" s="4">
         <v>1</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E32" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F32" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>104</v>
-      </c>
       <c r="G32" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H32" s="2"/>
     </row>
@@ -2384,22 +2381,22 @@
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C33" s="4">
         <v>1</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E33" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="F33" s="4" t="s">
-        <v>108</v>
-      </c>
       <c r="G33" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H33" s="2"/>
     </row>
@@ -2408,22 +2405,22 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C34" s="4">
         <v>2</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E34" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="F34" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="F34" s="4" t="s">
-        <v>112</v>
-      </c>
       <c r="G34" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H34" s="2"/>
     </row>
@@ -2432,22 +2429,22 @@
         <v>34</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C35" s="4">
         <v>1</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E35" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="F35" s="4" t="s">
-        <v>116</v>
-      </c>
       <c r="G35" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H35" s="2"/>
     </row>
@@ -2456,22 +2453,22 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C36" s="4">
         <v>3</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E36" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F36" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="F36" s="4" t="s">
-        <v>120</v>
-      </c>
       <c r="G36" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H36" s="2"/>
     </row>
@@ -2480,22 +2477,22 @@
         <v>36</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C37" s="4">
         <v>1</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E37" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F37" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="F37" s="4" t="s">
-        <v>124</v>
-      </c>
       <c r="G37" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H37" s="2"/>
     </row>
@@ -2504,22 +2501,22 @@
         <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C38" s="4">
         <v>1</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E38" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F38" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F38" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="G38" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H38" s="2"/>
     </row>
@@ -2528,22 +2525,22 @@
         <v>38</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C39" s="4">
         <v>1</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H39" s="2"/>
     </row>

</xml_diff>